<commit_message>
caso variable 1 dia
</commit_message>
<xml_diff>
--- a/data/data_chuqui_3mb_onboard_fixed/elmo_data.xlsx
+++ b/data/data_chuqui_3mb_onboard_fixed/elmo_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TECNO-MASTER\Desktop\Elmo_infrastructure_sizing_NP-\data\data_chuqui_3mb_onboard_fixed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{678E980D-974F-455D-8CEE-FCABD6DBA153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4136E517-E5A9-4AF4-BBF2-C5ACC1D926EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="1860" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Batteries" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1107" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1108" uniqueCount="392">
   <si>
     <t>id</t>
   </si>
@@ -1211,6 +1211,9 @@
   </si>
   <si>
     <t>Battery_swap</t>
+  </si>
+  <si>
+    <t>c</t>
   </si>
 </sst>
 </file>
@@ -4049,8 +4052,8 @@
       <c r="F3">
         <v>0</v>
       </c>
-      <c r="G3">
-        <v>24</v>
+      <c r="G3" t="s">
+        <v>391</v>
       </c>
       <c r="H3">
         <v>10000</v>

</xml_diff>